<commit_message>
adding validation ranges as stated in the current parameter list (xls)
</commit_message>
<xml_diff>
--- a/Documentation/VECTO Input Parameters.xlsx
+++ b/Documentation/VECTO Input Parameters.xlsx
@@ -6419,6 +6419,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="97" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6446,30 +6464,12 @@
     <xf numFmtId="0" fontId="31" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="97" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -6488,6 +6488,75 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="93" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="79" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="79" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="94" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="95" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -6495,75 +6564,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="79" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="93" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="79" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="94" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="95" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -6826,11 +6826,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="79575296"/>
-        <c:axId val="79688064"/>
+        <c:axId val="47579520"/>
+        <c:axId val="47581440"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="79575296"/>
+        <c:axId val="47579520"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="4000"/>
@@ -6860,14 +6860,14 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="79688064"/>
+        <c:crossAx val="47581440"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="2000"/>
         <c:minorUnit val="1000"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="79688064"/>
+        <c:axId val="47581440"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="2"/>
@@ -6897,7 +6897,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="79575296"/>
+        <c:crossAx val="47579520"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -7064,11 +7064,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="79431168"/>
-        <c:axId val="79433088"/>
+        <c:axId val="47332736"/>
+        <c:axId val="47339008"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="79431168"/>
+        <c:axId val="47332736"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="7"/>
@@ -7098,13 +7098,13 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="79433088"/>
+        <c:crossAx val="47339008"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="1"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="79433088"/>
+        <c:axId val="47339008"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7133,7 +7133,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="79431168"/>
+        <c:crossAx val="47332736"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -7304,11 +7304,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="79475072"/>
-        <c:axId val="79476992"/>
+        <c:axId val="47622400"/>
+        <c:axId val="96702848"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="79475072"/>
+        <c:axId val="47622400"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7336,12 +7336,12 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="79476992"/>
+        <c:crossAx val="96702848"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="79476992"/>
+        <c:axId val="96702848"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7370,7 +7370,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="79475072"/>
+        <c:crossAx val="47622400"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -7578,11 +7578,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="100633984"/>
-        <c:axId val="81544704"/>
+        <c:axId val="47269760"/>
+        <c:axId val="47284224"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="100633984"/>
+        <c:axId val="47269760"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7611,12 +7611,12 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="81544704"/>
+        <c:crossAx val="47284224"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="81544704"/>
+        <c:axId val="47284224"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7645,7 +7645,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="100633984"/>
+        <c:crossAx val="47269760"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -7822,8 +7822,8 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="100941824"/>
-        <c:axId val="100943744"/>
+        <c:axId val="49228032"/>
+        <c:axId val="49242496"/>
       </c:scatterChart>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
@@ -7939,11 +7939,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="100947840"/>
-        <c:axId val="100945920"/>
+        <c:axId val="49250688"/>
+        <c:axId val="49244416"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="100941824"/>
+        <c:axId val="49228032"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="1"/>
@@ -7973,12 +7973,12 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="100943744"/>
+        <c:crossAx val="49242496"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="100943744"/>
+        <c:axId val="49242496"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8007,12 +8007,12 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="100941824"/>
+        <c:crossAx val="49228032"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="100945920"/>
+        <c:axId val="49244416"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8040,12 +8040,12 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="100947840"/>
+        <c:crossAx val="49250688"/>
         <c:crosses val="max"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="100947840"/>
+        <c:axId val="49250688"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8055,7 +8055,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="100945920"/>
+        <c:crossAx val="49244416"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -8222,11 +8222,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="49424256"/>
-        <c:axId val="81690624"/>
+        <c:axId val="47251840"/>
+        <c:axId val="47253760"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="49424256"/>
+        <c:axId val="47251840"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8260,12 +8260,12 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="81690624"/>
+        <c:crossAx val="47253760"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="81690624"/>
+        <c:axId val="47253760"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8294,7 +8294,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="49424256"/>
+        <c:crossAx val="47251840"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -13114,7 +13114,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr codeName="Tabelle1"/>
+  <sheetPr codeName="Tabelle1">
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:T391"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -13133,7 +13135,9 @@
     <col min="13" max="13" width="11.42578125" style="71"/>
     <col min="14" max="14" width="17.42578125" style="74" customWidth="1"/>
     <col min="15" max="15" width="17.5703125" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="11.42578125" style="1"/>
+    <col min="16" max="19" width="11.42578125" style="1"/>
+    <col min="20" max="20" width="0" style="1" hidden="1" customWidth="1"/>
+    <col min="21" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -13143,21 +13147,21 @@
       </c>
     </row>
     <row r="2" spans="1:20" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="443" t="s">
+      <c r="B2" s="432" t="s">
         <v>280</v>
       </c>
-      <c r="C2" s="444"/>
-      <c r="D2" s="444"/>
-      <c r="E2" s="444"/>
-      <c r="F2" s="444"/>
-      <c r="G2" s="445"/>
-      <c r="H2" s="443" t="s">
+      <c r="C2" s="433"/>
+      <c r="D2" s="433"/>
+      <c r="E2" s="433"/>
+      <c r="F2" s="433"/>
+      <c r="G2" s="434"/>
+      <c r="H2" s="432" t="s">
         <v>279</v>
       </c>
-      <c r="I2" s="444"/>
-      <c r="J2" s="444"/>
-      <c r="K2" s="444"/>
-      <c r="L2" s="445"/>
+      <c r="I2" s="433"/>
+      <c r="J2" s="433"/>
+      <c r="K2" s="433"/>
+      <c r="L2" s="434"/>
       <c r="M2" s="331" t="s">
         <v>652</v>
       </c>
@@ -13389,7 +13393,7 @@
       <c r="C8" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="D8" s="442" t="s">
+      <c r="D8" s="431" t="s">
         <v>505</v>
       </c>
       <c r="E8" s="25" t="s">
@@ -13431,7 +13435,7 @@
       <c r="C9" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="442"/>
+      <c r="D9" s="431"/>
       <c r="E9" s="25" t="s">
         <v>241</v>
       </c>
@@ -13473,7 +13477,7 @@
       <c r="C10" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="442"/>
+      <c r="D10" s="431"/>
       <c r="E10" s="25" t="s">
         <v>418</v>
       </c>
@@ -13515,7 +13519,7 @@
       <c r="C11" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="442"/>
+      <c r="D11" s="431"/>
       <c r="E11" s="25" t="s">
         <v>417</v>
       </c>
@@ -13557,7 +13561,7 @@
       <c r="C12" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="D12" s="442"/>
+      <c r="D12" s="431"/>
       <c r="E12" s="25" t="s">
         <v>799</v>
       </c>
@@ -14183,7 +14187,7 @@
       <c r="C26" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D26" s="432" t="s">
+      <c r="D26" s="438" t="s">
         <v>492</v>
       </c>
       <c r="E26" s="25" t="s">
@@ -14227,7 +14231,7 @@
       <c r="C27" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D27" s="433"/>
+      <c r="D27" s="439"/>
       <c r="E27" s="25" t="s">
         <v>65</v>
       </c>
@@ -14269,7 +14273,7 @@
       <c r="C28" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D28" s="433"/>
+      <c r="D28" s="439"/>
       <c r="E28" s="25" t="s">
         <v>66</v>
       </c>
@@ -14311,7 +14315,7 @@
       <c r="C29" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D29" s="433"/>
+      <c r="D29" s="439"/>
       <c r="E29" s="25" t="s">
         <v>242</v>
       </c>
@@ -14353,7 +14357,7 @@
       <c r="C30" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D30" s="433"/>
+      <c r="D30" s="439"/>
       <c r="E30" s="25" t="s">
         <v>243</v>
       </c>
@@ -14395,7 +14399,7 @@
       <c r="C31" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="D31" s="434"/>
+      <c r="D31" s="440"/>
       <c r="E31" s="26" t="s">
         <v>244</v>
       </c>
@@ -14437,7 +14441,7 @@
       <c r="C32" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D32" s="435" t="s">
+      <c r="D32" s="441" t="s">
         <v>492</v>
       </c>
       <c r="E32" s="2" t="s">
@@ -14479,7 +14483,7 @@
       <c r="C33" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D33" s="436"/>
+      <c r="D33" s="442"/>
       <c r="E33" s="2" t="s">
         <v>246</v>
       </c>
@@ -14519,7 +14523,7 @@
       <c r="C34" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D34" s="436"/>
+      <c r="D34" s="442"/>
       <c r="E34" s="2" t="s">
         <v>247</v>
       </c>
@@ -14559,7 +14563,7 @@
       <c r="C35" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D35" s="436"/>
+      <c r="D35" s="442"/>
       <c r="E35" s="2" t="s">
         <v>248</v>
       </c>
@@ -14599,7 +14603,7 @@
       <c r="C36" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D36" s="436"/>
+      <c r="D36" s="442"/>
       <c r="E36" s="25" t="s">
         <v>249</v>
       </c>
@@ -14641,7 +14645,7 @@
       <c r="C37" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D37" s="436"/>
+      <c r="D37" s="442"/>
       <c r="E37" s="25" t="s">
         <v>424</v>
       </c>
@@ -14683,7 +14687,7 @@
       <c r="C38" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D38" s="436"/>
+      <c r="D38" s="442"/>
       <c r="E38" s="25" t="s">
         <v>262</v>
       </c>
@@ -14725,7 +14729,7 @@
       <c r="C39" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D39" s="436"/>
+      <c r="D39" s="442"/>
       <c r="E39" s="25" t="s">
         <v>425</v>
       </c>
@@ -14767,7 +14771,7 @@
       <c r="C40" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D40" s="436"/>
+      <c r="D40" s="442"/>
       <c r="E40" s="25" t="s">
         <v>426</v>
       </c>
@@ -14809,7 +14813,7 @@
       <c r="C41" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D41" s="436"/>
+      <c r="D41" s="442"/>
       <c r="E41" s="25" t="s">
         <v>427</v>
       </c>
@@ -14851,7 +14855,7 @@
       <c r="C42" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D42" s="436"/>
+      <c r="D42" s="442"/>
       <c r="E42" s="25" t="s">
         <v>428</v>
       </c>
@@ -14893,7 +14897,7 @@
       <c r="C43" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D43" s="436"/>
+      <c r="D43" s="442"/>
       <c r="E43" s="25" t="s">
         <v>429</v>
       </c>
@@ -14935,7 +14939,7 @@
       <c r="C44" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="D44" s="437"/>
+      <c r="D44" s="443"/>
       <c r="E44" s="26" t="s">
         <v>430</v>
       </c>
@@ -14977,7 +14981,7 @@
       <c r="C45" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="D45" s="432" t="s">
+      <c r="D45" s="438" t="s">
         <v>492</v>
       </c>
       <c r="E45" s="25" t="s">
@@ -15019,7 +15023,7 @@
       <c r="C46" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="D46" s="433"/>
+      <c r="D46" s="439"/>
       <c r="E46" s="25" t="s">
         <v>251</v>
       </c>
@@ -15059,7 +15063,7 @@
       <c r="C47" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="D47" s="434"/>
+      <c r="D47" s="440"/>
       <c r="E47" s="26" t="s">
         <v>252</v>
       </c>
@@ -15216,7 +15220,7 @@
       <c r="N50" s="74">
         <v>40000</v>
       </c>
-      <c r="O50" s="429" t="s">
+      <c r="O50" s="435" t="s">
         <v>452</v>
       </c>
       <c r="T50" s="341">
@@ -15262,7 +15266,7 @@
       <c r="N51" s="74">
         <v>40000</v>
       </c>
-      <c r="O51" s="429"/>
+      <c r="O51" s="435"/>
       <c r="T51" s="341">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -15306,7 +15310,7 @@
       <c r="N52" s="74">
         <v>40000</v>
       </c>
-      <c r="O52" s="429"/>
+      <c r="O52" s="435"/>
       <c r="T52" s="341">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -15348,7 +15352,7 @@
       <c r="N53" s="74">
         <v>40000</v>
       </c>
-      <c r="O53" s="429"/>
+      <c r="O53" s="435"/>
       <c r="T53" s="341">
         <f t="shared" si="0"/>
         <v>41</v>
@@ -15449,7 +15453,7 @@
       <c r="C56" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D56" s="438" t="s">
+      <c r="D56" s="430" t="s">
         <v>506</v>
       </c>
       <c r="E56" s="2" t="s">
@@ -15495,7 +15499,7 @@
       <c r="C57" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="D57" s="438"/>
+      <c r="D57" s="430"/>
       <c r="E57" s="25" t="s">
         <v>254</v>
       </c>
@@ -15535,7 +15539,7 @@
       <c r="C58" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D58" s="438"/>
+      <c r="D58" s="430"/>
       <c r="E58" s="2" t="s">
         <v>255</v>
       </c>
@@ -15575,7 +15579,7 @@
       <c r="C59" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D59" s="438"/>
+      <c r="D59" s="430"/>
       <c r="E59" s="2" t="s">
         <v>256</v>
       </c>
@@ -15615,7 +15619,7 @@
       <c r="C60" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="D60" s="438"/>
+      <c r="D60" s="430"/>
       <c r="E60" s="25" t="s">
         <v>444</v>
       </c>
@@ -15657,7 +15661,7 @@
       <c r="C61" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="D61" s="438"/>
+      <c r="D61" s="430"/>
       <c r="E61" s="25" t="s">
         <v>443</v>
       </c>
@@ -16003,7 +16007,7 @@
       <c r="C69" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D69" s="435" t="s">
+      <c r="D69" s="441" t="s">
         <v>492</v>
       </c>
       <c r="E69" s="2" t="s">
@@ -16045,7 +16049,7 @@
       <c r="C70" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D70" s="437"/>
+      <c r="D70" s="443"/>
       <c r="E70" s="4" t="s">
         <v>257</v>
       </c>
@@ -16085,7 +16089,7 @@
       <c r="C71" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="D71" s="435" t="s">
+      <c r="D71" s="441" t="s">
         <v>492</v>
       </c>
       <c r="E71" s="2" t="s">
@@ -16127,7 +16131,7 @@
       <c r="C72" s="4" t="s">
         <v>442</v>
       </c>
-      <c r="D72" s="437"/>
+      <c r="D72" s="443"/>
       <c r="E72" s="4" t="s">
         <v>259</v>
       </c>
@@ -16450,7 +16454,7 @@
       <c r="N79" s="74" t="s">
         <v>457</v>
       </c>
-      <c r="O79" s="439" t="s">
+      <c r="O79" s="444" t="s">
         <v>456</v>
       </c>
       <c r="T79" s="341">
@@ -16494,7 +16498,7 @@
       <c r="N80" s="74" t="s">
         <v>457</v>
       </c>
-      <c r="O80" s="439"/>
+      <c r="O80" s="444"/>
       <c r="T80" s="341">
         <f t="shared" si="1"/>
         <v>110</v>
@@ -16536,7 +16540,7 @@
       <c r="N81" s="78" t="s">
         <v>457</v>
       </c>
-      <c r="O81" s="440"/>
+      <c r="O81" s="445"/>
       <c r="T81" s="341">
         <f t="shared" si="1"/>
         <v>111</v>
@@ -16549,7 +16553,7 @@
       <c r="C82" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D82" s="435" t="s">
+      <c r="D82" s="441" t="s">
         <v>492</v>
       </c>
       <c r="E82" s="2" t="s">
@@ -16591,7 +16595,7 @@
       <c r="C83" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D83" s="436"/>
+      <c r="D83" s="442"/>
       <c r="E83" s="6" t="s">
         <v>263</v>
       </c>
@@ -16631,7 +16635,7 @@
       <c r="C84" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D84" s="436"/>
+      <c r="D84" s="442"/>
       <c r="E84" s="2" t="s">
         <v>264</v>
       </c>
@@ -16671,7 +16675,7 @@
       <c r="C85" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="D85" s="437"/>
+      <c r="D85" s="443"/>
       <c r="E85" s="26" t="s">
         <v>265</v>
       </c>
@@ -16713,7 +16717,7 @@
       <c r="C86" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D86" s="435" t="s">
+      <c r="D86" s="441" t="s">
         <v>492</v>
       </c>
       <c r="E86" s="2" t="s">
@@ -16755,7 +16759,7 @@
       <c r="C87" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D87" s="436"/>
+      <c r="D87" s="442"/>
       <c r="E87" s="6" t="s">
         <v>266</v>
       </c>
@@ -16795,7 +16799,7 @@
       <c r="C88" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D88" s="437"/>
+      <c r="D88" s="443"/>
       <c r="E88" s="4" t="s">
         <v>267</v>
       </c>
@@ -16921,7 +16925,7 @@
       <c r="C91" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="D91" s="442" t="s">
+      <c r="D91" s="431" t="s">
         <v>830</v>
       </c>
       <c r="E91" s="25" t="s">
@@ -16965,7 +16969,7 @@
       <c r="C92" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="D92" s="442"/>
+      <c r="D92" s="431"/>
       <c r="E92" s="25" t="s">
         <v>395</v>
       </c>
@@ -17009,7 +17013,7 @@
       <c r="C93" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="D93" s="442"/>
+      <c r="D93" s="431"/>
       <c r="E93" s="25" t="s">
         <v>268</v>
       </c>
@@ -17051,7 +17055,7 @@
       <c r="C94" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="D94" s="442"/>
+      <c r="D94" s="431"/>
       <c r="E94" s="25" t="s">
         <v>523</v>
       </c>
@@ -17093,7 +17097,7 @@
       <c r="C95" s="349" t="s">
         <v>53</v>
       </c>
-      <c r="D95" s="442"/>
+      <c r="D95" s="431"/>
       <c r="E95" s="349" t="s">
         <v>829</v>
       </c>
@@ -17656,7 +17660,7 @@
       <c r="N107" s="74" t="s">
         <v>12</v>
       </c>
-      <c r="O107" s="430" t="s">
+      <c r="O107" s="436" t="s">
         <v>468</v>
       </c>
       <c r="T107" s="341">
@@ -17700,7 +17704,7 @@
       <c r="N108" s="78">
         <v>10</v>
       </c>
-      <c r="O108" s="431"/>
+      <c r="O108" s="437"/>
       <c r="T108" s="341">
         <f t="shared" si="1"/>
         <v>127</v>
@@ -17851,7 +17855,7 @@
       <c r="C113" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D113" s="436" t="s">
+      <c r="D113" s="442" t="s">
         <v>492</v>
       </c>
       <c r="E113" s="2" t="s">
@@ -17895,7 +17899,7 @@
       <c r="C114" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D114" s="436"/>
+      <c r="D114" s="442"/>
       <c r="E114" s="2" t="s">
         <v>270</v>
       </c>
@@ -17937,7 +17941,7 @@
       <c r="C115" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D115" s="437"/>
+      <c r="D115" s="443"/>
       <c r="E115" s="4" t="s">
         <v>271</v>
       </c>
@@ -17979,7 +17983,7 @@
       <c r="C116" s="2" t="s">
         <v>653</v>
       </c>
-      <c r="D116" s="435" t="s">
+      <c r="D116" s="441" t="s">
         <v>492</v>
       </c>
       <c r="E116" s="2" t="s">
@@ -18021,7 +18025,7 @@
       <c r="C117" s="2" t="s">
         <v>653</v>
       </c>
-      <c r="D117" s="436"/>
+      <c r="D117" s="442"/>
       <c r="E117" s="2" t="s">
         <v>273</v>
       </c>
@@ -18061,7 +18065,7 @@
       <c r="C118" s="4" t="s">
         <v>653</v>
       </c>
-      <c r="D118" s="437"/>
+      <c r="D118" s="443"/>
       <c r="E118" s="4" t="s">
         <v>274</v>
       </c>
@@ -18173,7 +18177,7 @@
       <c r="C121" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D121" s="436" t="s">
+      <c r="D121" s="442" t="s">
         <v>492</v>
       </c>
       <c r="E121" s="2" t="s">
@@ -18204,7 +18208,7 @@
       <c r="N121" s="74">
         <v>1</v>
       </c>
-      <c r="O121" s="430" t="s">
+      <c r="O121" s="436" t="s">
         <v>469</v>
       </c>
       <c r="T121" s="341">
@@ -18219,7 +18223,7 @@
       <c r="C122" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D122" s="436"/>
+      <c r="D122" s="442"/>
       <c r="E122" s="2" t="s">
         <v>711</v>
       </c>
@@ -18248,7 +18252,7 @@
       <c r="N122" s="74" t="s">
         <v>465</v>
       </c>
-      <c r="O122" s="430"/>
+      <c r="O122" s="436"/>
       <c r="T122" s="341">
         <f t="shared" si="1"/>
         <v>100</v>
@@ -18261,7 +18265,7 @@
       <c r="C123" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D123" s="437"/>
+      <c r="D123" s="443"/>
       <c r="E123" s="4" t="s">
         <v>275</v>
       </c>
@@ -18290,7 +18294,7 @@
       <c r="N123" s="78" t="s">
         <v>450</v>
       </c>
-      <c r="O123" s="431"/>
+      <c r="O123" s="437"/>
       <c r="T123" s="341">
         <f t="shared" si="1"/>
         <v>101</v>
@@ -19415,7 +19419,7 @@
       <c r="C152" s="336" t="s">
         <v>52</v>
       </c>
-      <c r="D152" s="441" t="s">
+      <c r="D152" s="429" t="s">
         <v>517</v>
       </c>
       <c r="E152" s="336" t="s">
@@ -19457,7 +19461,7 @@
       <c r="C153" s="342" t="s">
         <v>52</v>
       </c>
-      <c r="D153" s="438"/>
+      <c r="D153" s="430"/>
       <c r="E153" s="342" t="s">
         <v>261</v>
       </c>
@@ -21074,11 +21078,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="D152:D153"/>
-    <mergeCell ref="D91:D95"/>
-    <mergeCell ref="D8:D12"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:L2"/>
     <mergeCell ref="O50:O53"/>
     <mergeCell ref="O121:O123"/>
     <mergeCell ref="D26:D31"/>
@@ -21094,6 +21093,11 @@
     <mergeCell ref="D56:D61"/>
     <mergeCell ref="O79:O81"/>
     <mergeCell ref="O107:O108"/>
+    <mergeCell ref="D152:D153"/>
+    <mergeCell ref="D91:D95"/>
+    <mergeCell ref="D8:D12"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:L2"/>
   </mergeCells>
   <conditionalFormatting sqref="H94 H96:H145 H4:H90 H151:H1028">
     <cfRule type="expression" dxfId="5" priority="9">
@@ -21126,7 +21130,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="8" scale="63" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -25496,10 +25500,10 @@
       <c r="B5" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C5" s="455" t="s">
+      <c r="C5" s="460" t="s">
         <v>668</v>
       </c>
-      <c r="D5" s="456"/>
+      <c r="D5" s="461"/>
       <c r="G5" s="36"/>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
@@ -25509,7 +25513,7 @@
       <c r="C6" s="303" t="s">
         <v>682</v>
       </c>
-      <c r="D6" s="452" t="s">
+      <c r="D6" s="475" t="s">
         <v>758</v>
       </c>
       <c r="G6" s="36"/>
@@ -25521,7 +25525,7 @@
       <c r="C7" s="80" t="s">
         <v>683</v>
       </c>
-      <c r="D7" s="453"/>
+      <c r="D7" s="476"/>
       <c r="G7" s="36"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
@@ -25531,7 +25535,7 @@
       <c r="C8" s="80" t="s">
         <v>684</v>
       </c>
-      <c r="D8" s="453"/>
+      <c r="D8" s="476"/>
       <c r="G8" s="36"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
@@ -25541,7 +25545,7 @@
       <c r="C9" s="80" t="s">
         <v>681</v>
       </c>
-      <c r="D9" s="453"/>
+      <c r="D9" s="476"/>
       <c r="G9" s="36"/>
     </row>
     <row r="10" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -25551,7 +25555,7 @@
       <c r="C10" s="227" t="s">
         <v>685</v>
       </c>
-      <c r="D10" s="454"/>
+      <c r="D10" s="477"/>
     </row>
     <row r="11" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="12" spans="2:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -25569,33 +25573,33 @@
       <c r="B13" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C13" s="455" t="s">
+      <c r="C13" s="460" t="s">
         <v>668</v>
       </c>
-      <c r="D13" s="456"/>
+      <c r="D13" s="461"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="304" t="s">
         <v>755</v>
       </c>
-      <c r="C14" s="457" t="s">
+      <c r="C14" s="462" t="s">
         <v>759</v>
       </c>
-      <c r="D14" s="458"/>
+      <c r="D14" s="463"/>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="223" t="s">
         <v>756</v>
       </c>
-      <c r="C15" s="459"/>
-      <c r="D15" s="460"/>
+      <c r="C15" s="464"/>
+      <c r="D15" s="465"/>
     </row>
     <row r="16" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="225" t="s">
         <v>757</v>
       </c>
-      <c r="C16" s="461"/>
-      <c r="D16" s="462"/>
+      <c r="C16" s="466"/>
+      <c r="D16" s="467"/>
     </row>
     <row r="17" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="18" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -25613,47 +25617,47 @@
       <c r="B19" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C19" s="455" t="s">
+      <c r="C19" s="460" t="s">
         <v>668</v>
       </c>
-      <c r="D19" s="456"/>
+      <c r="D19" s="461"/>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20" s="304" t="s">
         <v>760</v>
       </c>
-      <c r="C20" s="457" t="s">
+      <c r="C20" s="462" t="s">
         <v>796</v>
       </c>
-      <c r="D20" s="458"/>
+      <c r="D20" s="463"/>
     </row>
     <row r="21" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B21" s="223" t="s">
         <v>761</v>
       </c>
-      <c r="C21" s="459"/>
-      <c r="D21" s="460"/>
+      <c r="C21" s="464"/>
+      <c r="D21" s="465"/>
     </row>
     <row r="22" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B22" s="223" t="s">
         <v>762</v>
       </c>
-      <c r="C22" s="459"/>
-      <c r="D22" s="460"/>
+      <c r="C22" s="464"/>
+      <c r="D22" s="465"/>
     </row>
     <row r="23" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B23" s="223" t="s">
         <v>763</v>
       </c>
-      <c r="C23" s="459"/>
-      <c r="D23" s="460"/>
+      <c r="C23" s="464"/>
+      <c r="D23" s="465"/>
     </row>
     <row r="24" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="225" t="s">
         <v>764</v>
       </c>
-      <c r="C24" s="461"/>
-      <c r="D24" s="462"/>
+      <c r="C24" s="466"/>
+      <c r="D24" s="467"/>
     </row>
     <row r="25" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="26" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -25671,75 +25675,75 @@
       <c r="B27" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C27" s="455" t="s">
+      <c r="C27" s="460" t="s">
         <v>668</v>
       </c>
-      <c r="D27" s="456"/>
+      <c r="D27" s="461"/>
     </row>
     <row r="28" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B28" s="304" t="s">
         <v>765</v>
       </c>
-      <c r="C28" s="457" t="s">
+      <c r="C28" s="462" t="s">
         <v>797</v>
       </c>
-      <c r="D28" s="458"/>
+      <c r="D28" s="463"/>
     </row>
     <row r="29" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B29" s="223" t="s">
         <v>766</v>
       </c>
-      <c r="C29" s="459"/>
-      <c r="D29" s="460"/>
+      <c r="C29" s="464"/>
+      <c r="D29" s="465"/>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="223" t="s">
         <v>767</v>
       </c>
-      <c r="C30" s="459"/>
-      <c r="D30" s="460"/>
+      <c r="C30" s="464"/>
+      <c r="D30" s="465"/>
     </row>
     <row r="31" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B31" s="223" t="s">
         <v>768</v>
       </c>
-      <c r="C31" s="459"/>
-      <c r="D31" s="460"/>
+      <c r="C31" s="464"/>
+      <c r="D31" s="465"/>
     </row>
     <row r="32" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B32" s="223" t="s">
         <v>769</v>
       </c>
-      <c r="C32" s="459"/>
-      <c r="D32" s="460"/>
+      <c r="C32" s="464"/>
+      <c r="D32" s="465"/>
     </row>
     <row r="33" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B33" s="223" t="s">
         <v>770</v>
       </c>
-      <c r="C33" s="459"/>
-      <c r="D33" s="460"/>
+      <c r="C33" s="464"/>
+      <c r="D33" s="465"/>
     </row>
     <row r="34" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B34" s="223" t="s">
         <v>771</v>
       </c>
-      <c r="C34" s="459"/>
-      <c r="D34" s="460"/>
+      <c r="C34" s="464"/>
+      <c r="D34" s="465"/>
     </row>
     <row r="35" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B35" s="223" t="s">
         <v>772</v>
       </c>
-      <c r="C35" s="459"/>
-      <c r="D35" s="460"/>
+      <c r="C35" s="464"/>
+      <c r="D35" s="465"/>
     </row>
     <row r="36" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="225" t="s">
         <v>773</v>
       </c>
-      <c r="C36" s="461"/>
-      <c r="D36" s="462"/>
+      <c r="C36" s="466"/>
+      <c r="D36" s="467"/>
     </row>
     <row r="37" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="38" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -25757,10 +25761,10 @@
       <c r="B39" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C39" s="455" t="s">
+      <c r="C39" s="460" t="s">
         <v>668</v>
       </c>
-      <c r="D39" s="456"/>
+      <c r="D39" s="461"/>
     </row>
     <row r="40" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B40" s="304" t="s">
@@ -25769,7 +25773,7 @@
       <c r="C40" s="303" t="s">
         <v>779</v>
       </c>
-      <c r="D40" s="452" t="s">
+      <c r="D40" s="475" t="s">
         <v>780</v>
       </c>
     </row>
@@ -25780,7 +25784,7 @@
       <c r="C41" s="80" t="s">
         <v>781</v>
       </c>
-      <c r="D41" s="453"/>
+      <c r="D41" s="476"/>
     </row>
     <row r="42" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B42" s="223" t="s">
@@ -25789,7 +25793,7 @@
       <c r="C42" s="80" t="s">
         <v>782</v>
       </c>
-      <c r="D42" s="453"/>
+      <c r="D42" s="476"/>
     </row>
     <row r="43" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B43" s="225" t="s">
@@ -25798,7 +25802,7 @@
       <c r="C43" s="227" t="s">
         <v>778</v>
       </c>
-      <c r="D43" s="454"/>
+      <c r="D43" s="477"/>
     </row>
     <row r="44" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="45" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -25816,17 +25820,17 @@
       <c r="B46" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C46" s="455" t="s">
+      <c r="C46" s="460" t="s">
         <v>668</v>
       </c>
-      <c r="D46" s="456"/>
+      <c r="D46" s="461"/>
     </row>
     <row r="47" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B47" s="304" t="s">
         <v>783</v>
       </c>
       <c r="C47" s="303"/>
-      <c r="D47" s="452"/>
+      <c r="D47" s="475"/>
     </row>
     <row r="48" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B48" s="223" t="s">
@@ -25835,7 +25839,7 @@
       <c r="C48" s="80" t="s">
         <v>787</v>
       </c>
-      <c r="D48" s="453"/>
+      <c r="D48" s="476"/>
     </row>
     <row r="49" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B49" s="225" t="s">
@@ -25844,7 +25848,7 @@
       <c r="C49" s="227" t="s">
         <v>786</v>
       </c>
-      <c r="D49" s="454"/>
+      <c r="D49" s="477"/>
     </row>
     <row r="50" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="51" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -25862,10 +25866,10 @@
       <c r="B52" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C52" s="455" t="s">
+      <c r="C52" s="460" t="s">
         <v>668</v>
       </c>
-      <c r="D52" s="456"/>
+      <c r="D52" s="461"/>
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B53" s="304" t="s">
@@ -25874,7 +25878,7 @@
       <c r="C53" s="303" t="s">
         <v>793</v>
       </c>
-      <c r="D53" s="452" t="s">
+      <c r="D53" s="475" t="s">
         <v>795</v>
       </c>
     </row>
@@ -25885,7 +25889,7 @@
       <c r="C54" s="80" t="s">
         <v>792</v>
       </c>
-      <c r="D54" s="453"/>
+      <c r="D54" s="476"/>
     </row>
     <row r="55" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B55" s="223" t="s">
@@ -25894,14 +25898,14 @@
       <c r="C55" s="80" t="s">
         <v>794</v>
       </c>
-      <c r="D55" s="453"/>
+      <c r="D55" s="476"/>
     </row>
     <row r="56" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B56" s="225" t="s">
         <v>791</v>
       </c>
       <c r="C56" s="227"/>
-      <c r="D56" s="454"/>
+      <c r="D56" s="477"/>
     </row>
     <row r="57" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -25919,290 +25923,290 @@
       <c r="B59" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C59" s="455" t="s">
+      <c r="C59" s="460" t="s">
         <v>668</v>
       </c>
-      <c r="D59" s="456"/>
+      <c r="D59" s="461"/>
     </row>
     <row r="60" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B60" s="304" t="s">
         <v>841</v>
       </c>
-      <c r="C60" s="465"/>
-      <c r="D60" s="466"/>
+      <c r="C60" s="454"/>
+      <c r="D60" s="455"/>
     </row>
     <row r="61" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B61" s="223" t="s">
         <v>842</v>
       </c>
-      <c r="C61" s="467"/>
-      <c r="D61" s="468"/>
+      <c r="C61" s="456"/>
+      <c r="D61" s="457"/>
     </row>
     <row r="62" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B62" s="223" t="s">
         <v>843</v>
       </c>
-      <c r="C62" s="467"/>
-      <c r="D62" s="468"/>
+      <c r="C62" s="456"/>
+      <c r="D62" s="457"/>
     </row>
     <row r="63" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B63" s="223" t="s">
         <v>844</v>
       </c>
-      <c r="C63" s="467"/>
-      <c r="D63" s="468"/>
+      <c r="C63" s="456"/>
+      <c r="D63" s="457"/>
     </row>
     <row r="64" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B64" s="223" t="s">
         <v>845</v>
       </c>
-      <c r="C64" s="467"/>
-      <c r="D64" s="468"/>
+      <c r="C64" s="456"/>
+      <c r="D64" s="457"/>
     </row>
     <row r="65" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B65" s="223" t="s">
         <v>846</v>
       </c>
-      <c r="C65" s="467"/>
-      <c r="D65" s="468"/>
+      <c r="C65" s="456"/>
+      <c r="D65" s="457"/>
     </row>
     <row r="66" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B66" s="223" t="s">
         <v>847</v>
       </c>
-      <c r="C66" s="467"/>
-      <c r="D66" s="468"/>
+      <c r="C66" s="456"/>
+      <c r="D66" s="457"/>
     </row>
     <row r="67" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B67" s="223" t="s">
         <v>848</v>
       </c>
-      <c r="C67" s="467"/>
-      <c r="D67" s="468"/>
+      <c r="C67" s="456"/>
+      <c r="D67" s="457"/>
     </row>
     <row r="68" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B68" s="223" t="s">
         <v>849</v>
       </c>
-      <c r="C68" s="467"/>
-      <c r="D68" s="468"/>
+      <c r="C68" s="456"/>
+      <c r="D68" s="457"/>
     </row>
     <row r="69" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B69" s="223" t="s">
         <v>850</v>
       </c>
-      <c r="C69" s="467"/>
-      <c r="D69" s="468"/>
+      <c r="C69" s="456"/>
+      <c r="D69" s="457"/>
     </row>
     <row r="70" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B70" s="223" t="s">
         <v>851</v>
       </c>
-      <c r="C70" s="467"/>
-      <c r="D70" s="468"/>
+      <c r="C70" s="456"/>
+      <c r="D70" s="457"/>
     </row>
     <row r="71" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B71" s="223" t="s">
         <v>852</v>
       </c>
-      <c r="C71" s="467"/>
-      <c r="D71" s="468"/>
+      <c r="C71" s="456"/>
+      <c r="D71" s="457"/>
     </row>
     <row r="72" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B72" s="223" t="s">
         <v>853</v>
       </c>
-      <c r="C72" s="467"/>
-      <c r="D72" s="468"/>
+      <c r="C72" s="456"/>
+      <c r="D72" s="457"/>
     </row>
     <row r="73" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B73" s="223" t="s">
         <v>854</v>
       </c>
-      <c r="C73" s="467"/>
-      <c r="D73" s="468"/>
+      <c r="C73" s="456"/>
+      <c r="D73" s="457"/>
     </row>
     <row r="74" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B74" s="223" t="s">
         <v>855</v>
       </c>
-      <c r="C74" s="467"/>
-      <c r="D74" s="468"/>
+      <c r="C74" s="456"/>
+      <c r="D74" s="457"/>
     </row>
     <row r="75" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B75" s="223" t="s">
         <v>856</v>
       </c>
-      <c r="C75" s="467"/>
-      <c r="D75" s="468"/>
+      <c r="C75" s="456"/>
+      <c r="D75" s="457"/>
     </row>
     <row r="76" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B76" s="223" t="s">
         <v>857</v>
       </c>
-      <c r="C76" s="467"/>
-      <c r="D76" s="468"/>
+      <c r="C76" s="456"/>
+      <c r="D76" s="457"/>
     </row>
     <row r="77" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B77" s="223" t="s">
         <v>858</v>
       </c>
-      <c r="C77" s="467"/>
-      <c r="D77" s="468"/>
+      <c r="C77" s="456"/>
+      <c r="D77" s="457"/>
     </row>
     <row r="78" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B78" s="223" t="s">
         <v>859</v>
       </c>
-      <c r="C78" s="467"/>
-      <c r="D78" s="468"/>
+      <c r="C78" s="456"/>
+      <c r="D78" s="457"/>
     </row>
     <row r="79" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B79" s="223" t="s">
         <v>860</v>
       </c>
-      <c r="C79" s="467"/>
-      <c r="D79" s="468"/>
+      <c r="C79" s="456"/>
+      <c r="D79" s="457"/>
     </row>
     <row r="80" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B80" s="223" t="s">
         <v>861</v>
       </c>
-      <c r="C80" s="467"/>
-      <c r="D80" s="468"/>
+      <c r="C80" s="456"/>
+      <c r="D80" s="457"/>
     </row>
     <row r="81" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B81" s="223" t="s">
         <v>862</v>
       </c>
-      <c r="C81" s="467"/>
-      <c r="D81" s="468"/>
+      <c r="C81" s="456"/>
+      <c r="D81" s="457"/>
     </row>
     <row r="82" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B82" s="223" t="s">
         <v>863</v>
       </c>
-      <c r="C82" s="467"/>
-      <c r="D82" s="468"/>
+      <c r="C82" s="456"/>
+      <c r="D82" s="457"/>
     </row>
     <row r="83" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B83" s="223" t="s">
         <v>864</v>
       </c>
-      <c r="C83" s="467"/>
-      <c r="D83" s="468"/>
+      <c r="C83" s="456"/>
+      <c r="D83" s="457"/>
     </row>
     <row r="84" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B84" s="223" t="s">
         <v>865</v>
       </c>
-      <c r="C84" s="467"/>
-      <c r="D84" s="468"/>
+      <c r="C84" s="456"/>
+      <c r="D84" s="457"/>
     </row>
     <row r="85" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B85" s="223" t="s">
         <v>866</v>
       </c>
-      <c r="C85" s="467"/>
-      <c r="D85" s="468"/>
+      <c r="C85" s="456"/>
+      <c r="D85" s="457"/>
     </row>
     <row r="86" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B86" s="223" t="s">
         <v>867</v>
       </c>
-      <c r="C86" s="467"/>
-      <c r="D86" s="468"/>
+      <c r="C86" s="456"/>
+      <c r="D86" s="457"/>
     </row>
     <row r="87" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B87" s="223" t="s">
         <v>868</v>
       </c>
-      <c r="C87" s="467"/>
-      <c r="D87" s="468"/>
+      <c r="C87" s="456"/>
+      <c r="D87" s="457"/>
     </row>
     <row r="88" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B88" s="223" t="s">
         <v>869</v>
       </c>
-      <c r="C88" s="467"/>
-      <c r="D88" s="468"/>
+      <c r="C88" s="456"/>
+      <c r="D88" s="457"/>
     </row>
     <row r="89" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B89" s="223" t="s">
         <v>870</v>
       </c>
-      <c r="C89" s="467"/>
-      <c r="D89" s="468"/>
+      <c r="C89" s="456"/>
+      <c r="D89" s="457"/>
     </row>
     <row r="90" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B90" s="223" t="s">
         <v>871</v>
       </c>
-      <c r="C90" s="467"/>
-      <c r="D90" s="468"/>
+      <c r="C90" s="456"/>
+      <c r="D90" s="457"/>
     </row>
     <row r="91" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B91" s="223" t="s">
         <v>872</v>
       </c>
-      <c r="C91" s="467"/>
-      <c r="D91" s="468"/>
+      <c r="C91" s="456"/>
+      <c r="D91" s="457"/>
     </row>
     <row r="92" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B92" s="223" t="s">
         <v>873</v>
       </c>
-      <c r="C92" s="467"/>
-      <c r="D92" s="468"/>
+      <c r="C92" s="456"/>
+      <c r="D92" s="457"/>
     </row>
     <row r="93" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B93" s="223" t="s">
         <v>874</v>
       </c>
-      <c r="C93" s="467"/>
-      <c r="D93" s="468"/>
+      <c r="C93" s="456"/>
+      <c r="D93" s="457"/>
     </row>
     <row r="94" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B94" s="223" t="s">
         <v>875</v>
       </c>
-      <c r="C94" s="467"/>
-      <c r="D94" s="468"/>
+      <c r="C94" s="456"/>
+      <c r="D94" s="457"/>
     </row>
     <row r="95" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B95" s="223" t="s">
         <v>876</v>
       </c>
-      <c r="C95" s="467"/>
-      <c r="D95" s="468"/>
+      <c r="C95" s="456"/>
+      <c r="D95" s="457"/>
     </row>
     <row r="96" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B96" s="223" t="s">
         <v>877</v>
       </c>
-      <c r="C96" s="467"/>
-      <c r="D96" s="468"/>
+      <c r="C96" s="456"/>
+      <c r="D96" s="457"/>
     </row>
     <row r="97" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B97" s="223" t="s">
         <v>878</v>
       </c>
-      <c r="C97" s="467"/>
-      <c r="D97" s="468"/>
+      <c r="C97" s="456"/>
+      <c r="D97" s="457"/>
     </row>
     <row r="98" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B98" s="223" t="s">
         <v>879</v>
       </c>
-      <c r="C98" s="467"/>
-      <c r="D98" s="468"/>
+      <c r="C98" s="456"/>
+      <c r="D98" s="457"/>
     </row>
     <row r="99" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B99" s="225" t="s">
         <v>880</v>
       </c>
-      <c r="C99" s="469"/>
-      <c r="D99" s="470"/>
+      <c r="C99" s="458"/>
+      <c r="D99" s="459"/>
     </row>
     <row r="100" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="101" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -26220,38 +26224,38 @@
       <c r="B102" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C102" s="455" t="s">
+      <c r="C102" s="460" t="s">
         <v>668</v>
       </c>
-      <c r="D102" s="456"/>
+      <c r="D102" s="461"/>
     </row>
     <row r="103" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B103" s="304" t="s">
         <v>881</v>
       </c>
-      <c r="C103" s="457"/>
-      <c r="D103" s="458"/>
+      <c r="C103" s="462"/>
+      <c r="D103" s="463"/>
     </row>
     <row r="104" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B104" s="223" t="s">
         <v>882</v>
       </c>
-      <c r="C104" s="459"/>
-      <c r="D104" s="460"/>
+      <c r="C104" s="464"/>
+      <c r="D104" s="465"/>
     </row>
     <row r="105" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B105" s="223" t="s">
         <v>883</v>
       </c>
-      <c r="C105" s="459"/>
-      <c r="D105" s="460"/>
+      <c r="C105" s="464"/>
+      <c r="D105" s="465"/>
     </row>
     <row r="106" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B106" s="225" t="s">
         <v>884</v>
       </c>
-      <c r="C106" s="461"/>
-      <c r="D106" s="462"/>
+      <c r="C106" s="466"/>
+      <c r="D106" s="467"/>
     </row>
     <row r="107" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="108" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -26269,19 +26273,19 @@
       <c r="B109" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C109" s="455" t="s">
+      <c r="C109" s="460" t="s">
         <v>668</v>
       </c>
-      <c r="D109" s="456"/>
+      <c r="D109" s="461"/>
     </row>
     <row r="110" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B110" s="304" t="s">
         <v>803</v>
       </c>
-      <c r="C110" s="471" t="s">
+      <c r="C110" s="468" t="s">
         <v>682</v>
       </c>
-      <c r="D110" s="477" t="s">
+      <c r="D110" s="474" t="s">
         <v>817</v>
       </c>
     </row>
@@ -26289,94 +26293,94 @@
       <c r="B111" s="223" t="s">
         <v>804</v>
       </c>
-      <c r="C111" s="472"/>
-      <c r="D111" s="475"/>
+      <c r="C111" s="469"/>
+      <c r="D111" s="472"/>
     </row>
     <row r="112" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B112" s="223" t="s">
         <v>805</v>
       </c>
-      <c r="C112" s="472"/>
-      <c r="D112" s="475"/>
+      <c r="C112" s="469"/>
+      <c r="D112" s="472"/>
     </row>
     <row r="113" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B113" s="223" t="s">
         <v>806</v>
       </c>
-      <c r="C113" s="472"/>
-      <c r="D113" s="475"/>
+      <c r="C113" s="469"/>
+      <c r="D113" s="472"/>
     </row>
     <row r="114" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B114" s="223" t="s">
         <v>807</v>
       </c>
-      <c r="C114" s="472"/>
-      <c r="D114" s="475"/>
+      <c r="C114" s="469"/>
+      <c r="D114" s="472"/>
     </row>
     <row r="115" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B115" s="223" t="s">
         <v>808</v>
       </c>
-      <c r="C115" s="472"/>
-      <c r="D115" s="475"/>
+      <c r="C115" s="469"/>
+      <c r="D115" s="472"/>
     </row>
     <row r="116" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B116" s="223" t="s">
         <v>809</v>
       </c>
-      <c r="C116" s="472"/>
-      <c r="D116" s="475"/>
+      <c r="C116" s="469"/>
+      <c r="D116" s="472"/>
     </row>
     <row r="117" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B117" s="223" t="s">
         <v>810</v>
       </c>
-      <c r="C117" s="472"/>
-      <c r="D117" s="475"/>
+      <c r="C117" s="469"/>
+      <c r="D117" s="472"/>
     </row>
     <row r="118" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B118" s="223" t="s">
         <v>811</v>
       </c>
-      <c r="C118" s="472"/>
-      <c r="D118" s="475"/>
+      <c r="C118" s="469"/>
+      <c r="D118" s="472"/>
     </row>
     <row r="119" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B119" s="223" t="s">
         <v>812</v>
       </c>
-      <c r="C119" s="472"/>
-      <c r="D119" s="475"/>
+      <c r="C119" s="469"/>
+      <c r="D119" s="472"/>
     </row>
     <row r="120" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B120" s="223" t="s">
         <v>813</v>
       </c>
-      <c r="C120" s="473"/>
-      <c r="D120" s="475"/>
+      <c r="C120" s="470"/>
+      <c r="D120" s="472"/>
     </row>
     <row r="121" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B121" s="223" t="s">
         <v>814</v>
       </c>
-      <c r="C121" s="474" t="s">
+      <c r="C121" s="471" t="s">
         <v>683</v>
       </c>
-      <c r="D121" s="475"/>
+      <c r="D121" s="472"/>
     </row>
     <row r="122" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B122" s="223" t="s">
         <v>815</v>
       </c>
-      <c r="C122" s="475"/>
-      <c r="D122" s="475"/>
+      <c r="C122" s="472"/>
+      <c r="D122" s="472"/>
     </row>
     <row r="123" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B123" s="225" t="s">
         <v>816</v>
       </c>
-      <c r="C123" s="476"/>
-      <c r="D123" s="476"/>
+      <c r="C123" s="473"/>
+      <c r="D123" s="473"/>
     </row>
     <row r="124" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B124" s="240"/>
@@ -26398,36 +26402,22 @@
       <c r="B126" s="312" t="s">
         <v>819</v>
       </c>
-      <c r="C126" s="455" t="s">
+      <c r="C126" s="460" t="s">
         <v>668</v>
       </c>
-      <c r="D126" s="456"/>
+      <c r="D126" s="461"/>
     </row>
     <row r="127" spans="2:4" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B127" s="330" t="s">
         <v>818</v>
       </c>
-      <c r="C127" s="463" t="s">
+      <c r="C127" s="452" t="s">
         <v>820</v>
       </c>
-      <c r="D127" s="464"/>
+      <c r="D127" s="453"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="C127:D127"/>
-    <mergeCell ref="C60:D99"/>
-    <mergeCell ref="C102:D102"/>
-    <mergeCell ref="C103:D106"/>
-    <mergeCell ref="C109:D109"/>
-    <mergeCell ref="C126:D126"/>
-    <mergeCell ref="C110:C120"/>
-    <mergeCell ref="C121:C123"/>
-    <mergeCell ref="D110:D123"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="D47:D49"/>
-    <mergeCell ref="C52:D52"/>
-    <mergeCell ref="D53:D56"/>
-    <mergeCell ref="C59:D59"/>
     <mergeCell ref="D40:D43"/>
     <mergeCell ref="D6:D10"/>
     <mergeCell ref="C5:D5"/>
@@ -26438,6 +26428,20 @@
     <mergeCell ref="C27:D27"/>
     <mergeCell ref="C28:D36"/>
     <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="D47:D49"/>
+    <mergeCell ref="C52:D52"/>
+    <mergeCell ref="D53:D56"/>
+    <mergeCell ref="C59:D59"/>
+    <mergeCell ref="C127:D127"/>
+    <mergeCell ref="C60:D99"/>
+    <mergeCell ref="C102:D102"/>
+    <mergeCell ref="C103:D106"/>
+    <mergeCell ref="C109:D109"/>
+    <mergeCell ref="C126:D126"/>
+    <mergeCell ref="C110:C120"/>
+    <mergeCell ref="C121:C123"/>
+    <mergeCell ref="D110:D123"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated Input Parameters that Speedratio of TorqueConverter has to cover range from 0.0 to at least 2.2
</commit_message>
<xml_diff>
--- a/Documentation/VECTO Input Parameters.xlsx
+++ b/Documentation/VECTO Input Parameters.xlsx
@@ -1,8 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\michaelkrisper\Documents\vecto-sim\Documentation\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="-15" yWindow="45" windowWidth="14025" windowHeight="14430" tabRatio="856" activeTab="1"/>
   </bookViews>
@@ -32,7 +37,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Segment Table'!$D$7:$J$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'VECTO parameters'!$B$3:$O$149</definedName>
   </definedNames>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
@@ -42,7 +47,7 @@
     <author>Luz Raphael</author>
   </authors>
   <commentList>
-    <comment ref="AA9" authorId="0">
+    <comment ref="AA9" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -66,7 +71,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB9" authorId="0">
+    <comment ref="AB9" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -90,7 +95,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z10" authorId="0">
+    <comment ref="Z10" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -114,7 +119,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA10" authorId="0">
+    <comment ref="AA10" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -138,7 +143,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB10" authorId="0">
+    <comment ref="AB10" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -162,7 +167,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA11" authorId="0">
+    <comment ref="AA11" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -186,7 +191,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB11" authorId="0">
+    <comment ref="AB11" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -210,7 +215,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z12" authorId="0">
+    <comment ref="Z12" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -234,7 +239,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA12" authorId="0">
+    <comment ref="AA12" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -258,7 +263,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AC12" authorId="0">
+    <comment ref="AC12" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -282,7 +287,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z13" authorId="0">
+    <comment ref="Z13" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -306,7 +311,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA13" authorId="0">
+    <comment ref="AA13" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -330,7 +335,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z17" authorId="0">
+    <comment ref="Z17" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -354,7 +359,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA17" authorId="0">
+    <comment ref="AA17" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -378,7 +383,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AC17" authorId="0">
+    <comment ref="AC17" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -402,7 +407,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z18" authorId="0">
+    <comment ref="Z18" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -426,7 +431,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA18" authorId="0">
+    <comment ref="AA18" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -460,7 +465,7 @@
     <author>Luz Raphael</author>
   </authors>
   <commentList>
-    <comment ref="I4" authorId="0">
+    <comment ref="I4" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -490,7 +495,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2932" uniqueCount="987">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2933" uniqueCount="988">
   <si>
     <t>Parameter</t>
   </si>
@@ -3649,11 +3654,14 @@
   <si>
     <t>Select from {None, Primary (before gearbox), Secondary (after gearbox), Losses included in Gearbox}</t>
   </si>
+  <si>
+    <t>&gt;=2.2</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
@@ -6419,12 +6427,45 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="97" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -6437,39 +6478,6 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -6488,6 +6496,39 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="90" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="79" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="93" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -6512,30 +6553,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="79" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -6555,15 +6572,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="90" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -6686,9 +6694,9 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="de-DE"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -6722,9 +6730,12 @@
             <c:strRef>
               <c:f>'Eng Inertia'!$D$11:$D$12</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>Inertia including Flywheel and Clutch  [kgm²]</c:v>
+                  <c:v>Inertia including Flywheel and Clutch </c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>[kgm²]</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -6817,6 +6828,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-B91C-433E-9133-3CDBC3F6D43C}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -6915,9 +6931,9 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="de-DE"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -6999,6 +7015,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-EB7C-4EDA-9BC8-5955C0839AF8}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -7055,6 +7076,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-EB7C-4EDA-9BC8-5955C0839AF8}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -7170,9 +7196,9 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="de-DE"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7295,6 +7321,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-CD51-49D1-B29B-5690FC833FC4}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -7407,9 +7438,9 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="de-DE"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7502,6 +7533,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-31E1-4C99-AFE0-3D6E65D8ED8E}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -7569,6 +7605,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-31E1-4C99-AFE0-3D6E65D8ED8E}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -7682,9 +7723,9 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="de-DE"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7813,6 +7854,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9F10-420B-94F8-B27DB98E0305}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -7930,6 +7976,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-9F10-420B-94F8-B27DB98E0305}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -8092,9 +8143,9 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="de-DE"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -8213,6 +8264,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-15DA-4250-B128-B314A8F818AA}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -8582,9 +8638,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Larissa">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
-    <a:clrScheme name="Larissa">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -8622,9 +8678,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Larissa">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8659,7 +8715,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -8694,7 +8750,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Larissa">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -13147,21 +13203,21 @@
       </c>
     </row>
     <row r="2" spans="1:20" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="432" t="s">
+      <c r="B2" s="443" t="s">
         <v>280</v>
       </c>
-      <c r="C2" s="433"/>
-      <c r="D2" s="433"/>
-      <c r="E2" s="433"/>
-      <c r="F2" s="433"/>
-      <c r="G2" s="434"/>
-      <c r="H2" s="432" t="s">
+      <c r="C2" s="444"/>
+      <c r="D2" s="444"/>
+      <c r="E2" s="444"/>
+      <c r="F2" s="444"/>
+      <c r="G2" s="445"/>
+      <c r="H2" s="443" t="s">
         <v>279</v>
       </c>
-      <c r="I2" s="433"/>
-      <c r="J2" s="433"/>
-      <c r="K2" s="433"/>
-      <c r="L2" s="434"/>
+      <c r="I2" s="444"/>
+      <c r="J2" s="444"/>
+      <c r="K2" s="444"/>
+      <c r="L2" s="445"/>
       <c r="M2" s="331" t="s">
         <v>652</v>
       </c>
@@ -13393,7 +13449,7 @@
       <c r="C8" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="D8" s="431" t="s">
+      <c r="D8" s="442" t="s">
         <v>505</v>
       </c>
       <c r="E8" s="25" t="s">
@@ -13435,7 +13491,7 @@
       <c r="C9" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="431"/>
+      <c r="D9" s="442"/>
       <c r="E9" s="25" t="s">
         <v>241</v>
       </c>
@@ -13477,7 +13533,7 @@
       <c r="C10" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="431"/>
+      <c r="D10" s="442"/>
       <c r="E10" s="25" t="s">
         <v>418</v>
       </c>
@@ -13519,7 +13575,7 @@
       <c r="C11" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="431"/>
+      <c r="D11" s="442"/>
       <c r="E11" s="25" t="s">
         <v>417</v>
       </c>
@@ -13561,7 +13617,7 @@
       <c r="C12" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="D12" s="431"/>
+      <c r="D12" s="442"/>
       <c r="E12" s="25" t="s">
         <v>799</v>
       </c>
@@ -14187,7 +14243,7 @@
       <c r="C26" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D26" s="438" t="s">
+      <c r="D26" s="432" t="s">
         <v>492</v>
       </c>
       <c r="E26" s="25" t="s">
@@ -14231,7 +14287,7 @@
       <c r="C27" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D27" s="439"/>
+      <c r="D27" s="433"/>
       <c r="E27" s="25" t="s">
         <v>65</v>
       </c>
@@ -14273,7 +14329,7 @@
       <c r="C28" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D28" s="439"/>
+      <c r="D28" s="433"/>
       <c r="E28" s="25" t="s">
         <v>66</v>
       </c>
@@ -14315,7 +14371,7 @@
       <c r="C29" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D29" s="439"/>
+      <c r="D29" s="433"/>
       <c r="E29" s="25" t="s">
         <v>242</v>
       </c>
@@ -14357,7 +14413,7 @@
       <c r="C30" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="D30" s="439"/>
+      <c r="D30" s="433"/>
       <c r="E30" s="25" t="s">
         <v>243</v>
       </c>
@@ -14399,7 +14455,7 @@
       <c r="C31" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="D31" s="440"/>
+      <c r="D31" s="434"/>
       <c r="E31" s="26" t="s">
         <v>244</v>
       </c>
@@ -14441,7 +14497,7 @@
       <c r="C32" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D32" s="441" t="s">
+      <c r="D32" s="435" t="s">
         <v>492</v>
       </c>
       <c r="E32" s="2" t="s">
@@ -14483,7 +14539,7 @@
       <c r="C33" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D33" s="442"/>
+      <c r="D33" s="436"/>
       <c r="E33" s="2" t="s">
         <v>246</v>
       </c>
@@ -14523,7 +14579,7 @@
       <c r="C34" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D34" s="442"/>
+      <c r="D34" s="436"/>
       <c r="E34" s="2" t="s">
         <v>247</v>
       </c>
@@ -14563,7 +14619,7 @@
       <c r="C35" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D35" s="442"/>
+      <c r="D35" s="436"/>
       <c r="E35" s="2" t="s">
         <v>248</v>
       </c>
@@ -14603,7 +14659,7 @@
       <c r="C36" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D36" s="442"/>
+      <c r="D36" s="436"/>
       <c r="E36" s="25" t="s">
         <v>249</v>
       </c>
@@ -14645,7 +14701,7 @@
       <c r="C37" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D37" s="442"/>
+      <c r="D37" s="436"/>
       <c r="E37" s="25" t="s">
         <v>424</v>
       </c>
@@ -14687,7 +14743,7 @@
       <c r="C38" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D38" s="442"/>
+      <c r="D38" s="436"/>
       <c r="E38" s="25" t="s">
         <v>262</v>
       </c>
@@ -14729,7 +14785,7 @@
       <c r="C39" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D39" s="442"/>
+      <c r="D39" s="436"/>
       <c r="E39" s="25" t="s">
         <v>425</v>
       </c>
@@ -14771,7 +14827,7 @@
       <c r="C40" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D40" s="442"/>
+      <c r="D40" s="436"/>
       <c r="E40" s="25" t="s">
         <v>426</v>
       </c>
@@ -14813,7 +14869,7 @@
       <c r="C41" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D41" s="442"/>
+      <c r="D41" s="436"/>
       <c r="E41" s="25" t="s">
         <v>427</v>
       </c>
@@ -14855,7 +14911,7 @@
       <c r="C42" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D42" s="442"/>
+      <c r="D42" s="436"/>
       <c r="E42" s="25" t="s">
         <v>428</v>
       </c>
@@ -14897,7 +14953,7 @@
       <c r="C43" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D43" s="442"/>
+      <c r="D43" s="436"/>
       <c r="E43" s="25" t="s">
         <v>429</v>
       </c>
@@ -14939,7 +14995,7 @@
       <c r="C44" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="D44" s="443"/>
+      <c r="D44" s="437"/>
       <c r="E44" s="26" t="s">
         <v>430</v>
       </c>
@@ -14981,7 +15037,7 @@
       <c r="C45" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="D45" s="438" t="s">
+      <c r="D45" s="432" t="s">
         <v>492</v>
       </c>
       <c r="E45" s="25" t="s">
@@ -15023,7 +15079,7 @@
       <c r="C46" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="D46" s="439"/>
+      <c r="D46" s="433"/>
       <c r="E46" s="25" t="s">
         <v>251</v>
       </c>
@@ -15063,7 +15119,7 @@
       <c r="C47" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="D47" s="440"/>
+      <c r="D47" s="434"/>
       <c r="E47" s="26" t="s">
         <v>252</v>
       </c>
@@ -15220,7 +15276,7 @@
       <c r="N50" s="74">
         <v>40000</v>
       </c>
-      <c r="O50" s="435" t="s">
+      <c r="O50" s="429" t="s">
         <v>452</v>
       </c>
       <c r="T50" s="341">
@@ -15266,7 +15322,7 @@
       <c r="N51" s="74">
         <v>40000</v>
       </c>
-      <c r="O51" s="435"/>
+      <c r="O51" s="429"/>
       <c r="T51" s="341">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -15310,7 +15366,7 @@
       <c r="N52" s="74">
         <v>40000</v>
       </c>
-      <c r="O52" s="435"/>
+      <c r="O52" s="429"/>
       <c r="T52" s="341">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -15352,7 +15408,7 @@
       <c r="N53" s="74">
         <v>40000</v>
       </c>
-      <c r="O53" s="435"/>
+      <c r="O53" s="429"/>
       <c r="T53" s="341">
         <f t="shared" si="0"/>
         <v>41</v>
@@ -15453,7 +15509,7 @@
       <c r="C56" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D56" s="430" t="s">
+      <c r="D56" s="438" t="s">
         <v>506</v>
       </c>
       <c r="E56" s="2" t="s">
@@ -15499,7 +15555,7 @@
       <c r="C57" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="D57" s="430"/>
+      <c r="D57" s="438"/>
       <c r="E57" s="25" t="s">
         <v>254</v>
       </c>
@@ -15539,7 +15595,7 @@
       <c r="C58" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D58" s="430"/>
+      <c r="D58" s="438"/>
       <c r="E58" s="2" t="s">
         <v>255</v>
       </c>
@@ -15579,7 +15635,7 @@
       <c r="C59" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D59" s="430"/>
+      <c r="D59" s="438"/>
       <c r="E59" s="2" t="s">
         <v>256</v>
       </c>
@@ -15619,7 +15675,7 @@
       <c r="C60" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="D60" s="430"/>
+      <c r="D60" s="438"/>
       <c r="E60" s="25" t="s">
         <v>444</v>
       </c>
@@ -15661,7 +15717,7 @@
       <c r="C61" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="D61" s="430"/>
+      <c r="D61" s="438"/>
       <c r="E61" s="25" t="s">
         <v>443</v>
       </c>
@@ -16007,7 +16063,7 @@
       <c r="C69" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D69" s="441" t="s">
+      <c r="D69" s="435" t="s">
         <v>492</v>
       </c>
       <c r="E69" s="2" t="s">
@@ -16049,7 +16105,7 @@
       <c r="C70" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D70" s="443"/>
+      <c r="D70" s="437"/>
       <c r="E70" s="4" t="s">
         <v>257</v>
       </c>
@@ -16089,7 +16145,7 @@
       <c r="C71" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="D71" s="441" t="s">
+      <c r="D71" s="435" t="s">
         <v>492</v>
       </c>
       <c r="E71" s="2" t="s">
@@ -16131,7 +16187,7 @@
       <c r="C72" s="4" t="s">
         <v>442</v>
       </c>
-      <c r="D72" s="443"/>
+      <c r="D72" s="437"/>
       <c r="E72" s="4" t="s">
         <v>259</v>
       </c>
@@ -16454,7 +16510,7 @@
       <c r="N79" s="74" t="s">
         <v>457</v>
       </c>
-      <c r="O79" s="444" t="s">
+      <c r="O79" s="439" t="s">
         <v>456</v>
       </c>
       <c r="T79" s="341">
@@ -16498,7 +16554,7 @@
       <c r="N80" s="74" t="s">
         <v>457</v>
       </c>
-      <c r="O80" s="444"/>
+      <c r="O80" s="439"/>
       <c r="T80" s="341">
         <f t="shared" si="1"/>
         <v>110</v>
@@ -16540,7 +16596,7 @@
       <c r="N81" s="78" t="s">
         <v>457</v>
       </c>
-      <c r="O81" s="445"/>
+      <c r="O81" s="440"/>
       <c r="T81" s="341">
         <f t="shared" si="1"/>
         <v>111</v>
@@ -16553,7 +16609,7 @@
       <c r="C82" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D82" s="441" t="s">
+      <c r="D82" s="435" t="s">
         <v>492</v>
       </c>
       <c r="E82" s="2" t="s">
@@ -16595,7 +16651,7 @@
       <c r="C83" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D83" s="442"/>
+      <c r="D83" s="436"/>
       <c r="E83" s="6" t="s">
         <v>263</v>
       </c>
@@ -16635,7 +16691,7 @@
       <c r="C84" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D84" s="442"/>
+      <c r="D84" s="436"/>
       <c r="E84" s="2" t="s">
         <v>264</v>
       </c>
@@ -16675,7 +16731,7 @@
       <c r="C85" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="D85" s="443"/>
+      <c r="D85" s="437"/>
       <c r="E85" s="26" t="s">
         <v>265</v>
       </c>
@@ -16717,7 +16773,7 @@
       <c r="C86" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D86" s="441" t="s">
+      <c r="D86" s="435" t="s">
         <v>492</v>
       </c>
       <c r="E86" s="2" t="s">
@@ -16759,7 +16815,7 @@
       <c r="C87" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D87" s="442"/>
+      <c r="D87" s="436"/>
       <c r="E87" s="6" t="s">
         <v>266</v>
       </c>
@@ -16799,7 +16855,7 @@
       <c r="C88" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D88" s="443"/>
+      <c r="D88" s="437"/>
       <c r="E88" s="4" t="s">
         <v>267</v>
       </c>
@@ -16925,7 +16981,7 @@
       <c r="C91" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="D91" s="431" t="s">
+      <c r="D91" s="442" t="s">
         <v>830</v>
       </c>
       <c r="E91" s="25" t="s">
@@ -16969,7 +17025,7 @@
       <c r="C92" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="D92" s="431"/>
+      <c r="D92" s="442"/>
       <c r="E92" s="25" t="s">
         <v>395</v>
       </c>
@@ -17013,7 +17069,7 @@
       <c r="C93" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="D93" s="431"/>
+      <c r="D93" s="442"/>
       <c r="E93" s="25" t="s">
         <v>268</v>
       </c>
@@ -17055,7 +17111,7 @@
       <c r="C94" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="D94" s="431"/>
+      <c r="D94" s="442"/>
       <c r="E94" s="25" t="s">
         <v>523</v>
       </c>
@@ -17097,7 +17153,7 @@
       <c r="C95" s="349" t="s">
         <v>53</v>
       </c>
-      <c r="D95" s="431"/>
+      <c r="D95" s="442"/>
       <c r="E95" s="349" t="s">
         <v>829</v>
       </c>
@@ -17660,7 +17716,7 @@
       <c r="N107" s="74" t="s">
         <v>12</v>
       </c>
-      <c r="O107" s="436" t="s">
+      <c r="O107" s="430" t="s">
         <v>468</v>
       </c>
       <c r="T107" s="341">
@@ -17704,7 +17760,7 @@
       <c r="N108" s="78">
         <v>10</v>
       </c>
-      <c r="O108" s="437"/>
+      <c r="O108" s="431"/>
       <c r="T108" s="341">
         <f t="shared" si="1"/>
         <v>127</v>
@@ -17855,7 +17911,7 @@
       <c r="C113" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D113" s="442" t="s">
+      <c r="D113" s="436" t="s">
         <v>492</v>
       </c>
       <c r="E113" s="2" t="s">
@@ -17899,7 +17955,7 @@
       <c r="C114" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D114" s="442"/>
+      <c r="D114" s="436"/>
       <c r="E114" s="2" t="s">
         <v>270</v>
       </c>
@@ -17941,7 +17997,7 @@
       <c r="C115" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D115" s="443"/>
+      <c r="D115" s="437"/>
       <c r="E115" s="4" t="s">
         <v>271</v>
       </c>
@@ -17983,7 +18039,7 @@
       <c r="C116" s="2" t="s">
         <v>653</v>
       </c>
-      <c r="D116" s="441" t="s">
+      <c r="D116" s="435" t="s">
         <v>492</v>
       </c>
       <c r="E116" s="2" t="s">
@@ -18025,7 +18081,7 @@
       <c r="C117" s="2" t="s">
         <v>653</v>
       </c>
-      <c r="D117" s="442"/>
+      <c r="D117" s="436"/>
       <c r="E117" s="2" t="s">
         <v>273</v>
       </c>
@@ -18065,7 +18121,7 @@
       <c r="C118" s="4" t="s">
         <v>653</v>
       </c>
-      <c r="D118" s="443"/>
+      <c r="D118" s="437"/>
       <c r="E118" s="4" t="s">
         <v>274</v>
       </c>
@@ -18177,7 +18233,7 @@
       <c r="C121" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D121" s="442" t="s">
+      <c r="D121" s="436" t="s">
         <v>492</v>
       </c>
       <c r="E121" s="2" t="s">
@@ -18205,10 +18261,10 @@
       <c r="M121" s="70">
         <v>0</v>
       </c>
-      <c r="N121" s="74">
-        <v>1</v>
-      </c>
-      <c r="O121" s="436" t="s">
+      <c r="N121" s="74" t="s">
+        <v>987</v>
+      </c>
+      <c r="O121" s="430" t="s">
         <v>469</v>
       </c>
       <c r="T121" s="341">
@@ -18223,7 +18279,7 @@
       <c r="C122" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D122" s="442"/>
+      <c r="D122" s="436"/>
       <c r="E122" s="2" t="s">
         <v>711</v>
       </c>
@@ -18252,7 +18308,7 @@
       <c r="N122" s="74" t="s">
         <v>465</v>
       </c>
-      <c r="O122" s="436"/>
+      <c r="O122" s="430"/>
       <c r="T122" s="341">
         <f t="shared" si="1"/>
         <v>100</v>
@@ -18265,7 +18321,7 @@
       <c r="C123" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D123" s="443"/>
+      <c r="D123" s="437"/>
       <c r="E123" s="4" t="s">
         <v>275</v>
       </c>
@@ -18294,7 +18350,7 @@
       <c r="N123" s="78" t="s">
         <v>450</v>
       </c>
-      <c r="O123" s="437"/>
+      <c r="O123" s="431"/>
       <c r="T123" s="341">
         <f t="shared" si="1"/>
         <v>101</v>
@@ -19419,7 +19475,7 @@
       <c r="C152" s="336" t="s">
         <v>52</v>
       </c>
-      <c r="D152" s="429" t="s">
+      <c r="D152" s="441" t="s">
         <v>517</v>
       </c>
       <c r="E152" s="336" t="s">
@@ -19461,7 +19517,7 @@
       <c r="C153" s="342" t="s">
         <v>52</v>
       </c>
-      <c r="D153" s="430"/>
+      <c r="D153" s="438"/>
       <c r="E153" s="342" t="s">
         <v>261</v>
       </c>
@@ -21078,6 +21134,11 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="D152:D153"/>
+    <mergeCell ref="D91:D95"/>
+    <mergeCell ref="D8:D12"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:L2"/>
     <mergeCell ref="O50:O53"/>
     <mergeCell ref="O121:O123"/>
     <mergeCell ref="D26:D31"/>
@@ -21093,11 +21154,6 @@
     <mergeCell ref="D56:D61"/>
     <mergeCell ref="O79:O81"/>
     <mergeCell ref="O107:O108"/>
-    <mergeCell ref="D152:D153"/>
-    <mergeCell ref="D91:D95"/>
-    <mergeCell ref="D8:D12"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:L2"/>
   </mergeCells>
   <conditionalFormatting sqref="H94 H96:H145 H4:H90 H151:H1028">
     <cfRule type="expression" dxfId="5" priority="9">
@@ -25500,10 +25556,10 @@
       <c r="B5" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C5" s="460" t="s">
+      <c r="C5" s="455" t="s">
         <v>668</v>
       </c>
-      <c r="D5" s="461"/>
+      <c r="D5" s="456"/>
       <c r="G5" s="36"/>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
@@ -25513,7 +25569,7 @@
       <c r="C6" s="303" t="s">
         <v>682</v>
       </c>
-      <c r="D6" s="475" t="s">
+      <c r="D6" s="452" t="s">
         <v>758</v>
       </c>
       <c r="G6" s="36"/>
@@ -25525,7 +25581,7 @@
       <c r="C7" s="80" t="s">
         <v>683</v>
       </c>
-      <c r="D7" s="476"/>
+      <c r="D7" s="453"/>
       <c r="G7" s="36"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
@@ -25535,7 +25591,7 @@
       <c r="C8" s="80" t="s">
         <v>684</v>
       </c>
-      <c r="D8" s="476"/>
+      <c r="D8" s="453"/>
       <c r="G8" s="36"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
@@ -25545,7 +25601,7 @@
       <c r="C9" s="80" t="s">
         <v>681</v>
       </c>
-      <c r="D9" s="476"/>
+      <c r="D9" s="453"/>
       <c r="G9" s="36"/>
     </row>
     <row r="10" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -25555,7 +25611,7 @@
       <c r="C10" s="227" t="s">
         <v>685</v>
       </c>
-      <c r="D10" s="477"/>
+      <c r="D10" s="454"/>
     </row>
     <row r="11" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="12" spans="2:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -25573,33 +25629,33 @@
       <c r="B13" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C13" s="460" t="s">
+      <c r="C13" s="455" t="s">
         <v>668</v>
       </c>
-      <c r="D13" s="461"/>
+      <c r="D13" s="456"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="304" t="s">
         <v>755</v>
       </c>
-      <c r="C14" s="462" t="s">
+      <c r="C14" s="457" t="s">
         <v>759</v>
       </c>
-      <c r="D14" s="463"/>
+      <c r="D14" s="458"/>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="223" t="s">
         <v>756</v>
       </c>
-      <c r="C15" s="464"/>
-      <c r="D15" s="465"/>
+      <c r="C15" s="459"/>
+      <c r="D15" s="460"/>
     </row>
     <row r="16" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="225" t="s">
         <v>757</v>
       </c>
-      <c r="C16" s="466"/>
-      <c r="D16" s="467"/>
+      <c r="C16" s="461"/>
+      <c r="D16" s="462"/>
     </row>
     <row r="17" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="18" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -25617,47 +25673,47 @@
       <c r="B19" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C19" s="460" t="s">
+      <c r="C19" s="455" t="s">
         <v>668</v>
       </c>
-      <c r="D19" s="461"/>
+      <c r="D19" s="456"/>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20" s="304" t="s">
         <v>760</v>
       </c>
-      <c r="C20" s="462" t="s">
+      <c r="C20" s="457" t="s">
         <v>796</v>
       </c>
-      <c r="D20" s="463"/>
+      <c r="D20" s="458"/>
     </row>
     <row r="21" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B21" s="223" t="s">
         <v>761</v>
       </c>
-      <c r="C21" s="464"/>
-      <c r="D21" s="465"/>
+      <c r="C21" s="459"/>
+      <c r="D21" s="460"/>
     </row>
     <row r="22" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B22" s="223" t="s">
         <v>762</v>
       </c>
-      <c r="C22" s="464"/>
-      <c r="D22" s="465"/>
+      <c r="C22" s="459"/>
+      <c r="D22" s="460"/>
     </row>
     <row r="23" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B23" s="223" t="s">
         <v>763</v>
       </c>
-      <c r="C23" s="464"/>
-      <c r="D23" s="465"/>
+      <c r="C23" s="459"/>
+      <c r="D23" s="460"/>
     </row>
     <row r="24" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="225" t="s">
         <v>764</v>
       </c>
-      <c r="C24" s="466"/>
-      <c r="D24" s="467"/>
+      <c r="C24" s="461"/>
+      <c r="D24" s="462"/>
     </row>
     <row r="25" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="26" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -25675,75 +25731,75 @@
       <c r="B27" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C27" s="460" t="s">
+      <c r="C27" s="455" t="s">
         <v>668</v>
       </c>
-      <c r="D27" s="461"/>
+      <c r="D27" s="456"/>
     </row>
     <row r="28" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B28" s="304" t="s">
         <v>765</v>
       </c>
-      <c r="C28" s="462" t="s">
+      <c r="C28" s="457" t="s">
         <v>797</v>
       </c>
-      <c r="D28" s="463"/>
+      <c r="D28" s="458"/>
     </row>
     <row r="29" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B29" s="223" t="s">
         <v>766</v>
       </c>
-      <c r="C29" s="464"/>
-      <c r="D29" s="465"/>
+      <c r="C29" s="459"/>
+      <c r="D29" s="460"/>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="223" t="s">
         <v>767</v>
       </c>
-      <c r="C30" s="464"/>
-      <c r="D30" s="465"/>
+      <c r="C30" s="459"/>
+      <c r="D30" s="460"/>
     </row>
     <row r="31" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B31" s="223" t="s">
         <v>768</v>
       </c>
-      <c r="C31" s="464"/>
-      <c r="D31" s="465"/>
+      <c r="C31" s="459"/>
+      <c r="D31" s="460"/>
     </row>
     <row r="32" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B32" s="223" t="s">
         <v>769</v>
       </c>
-      <c r="C32" s="464"/>
-      <c r="D32" s="465"/>
+      <c r="C32" s="459"/>
+      <c r="D32" s="460"/>
     </row>
     <row r="33" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B33" s="223" t="s">
         <v>770</v>
       </c>
-      <c r="C33" s="464"/>
-      <c r="D33" s="465"/>
+      <c r="C33" s="459"/>
+      <c r="D33" s="460"/>
     </row>
     <row r="34" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B34" s="223" t="s">
         <v>771</v>
       </c>
-      <c r="C34" s="464"/>
-      <c r="D34" s="465"/>
+      <c r="C34" s="459"/>
+      <c r="D34" s="460"/>
     </row>
     <row r="35" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B35" s="223" t="s">
         <v>772</v>
       </c>
-      <c r="C35" s="464"/>
-      <c r="D35" s="465"/>
+      <c r="C35" s="459"/>
+      <c r="D35" s="460"/>
     </row>
     <row r="36" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="225" t="s">
         <v>773</v>
       </c>
-      <c r="C36" s="466"/>
-      <c r="D36" s="467"/>
+      <c r="C36" s="461"/>
+      <c r="D36" s="462"/>
     </row>
     <row r="37" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="38" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -25761,10 +25817,10 @@
       <c r="B39" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C39" s="460" t="s">
+      <c r="C39" s="455" t="s">
         <v>668</v>
       </c>
-      <c r="D39" s="461"/>
+      <c r="D39" s="456"/>
     </row>
     <row r="40" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B40" s="304" t="s">
@@ -25773,7 +25829,7 @@
       <c r="C40" s="303" t="s">
         <v>779</v>
       </c>
-      <c r="D40" s="475" t="s">
+      <c r="D40" s="452" t="s">
         <v>780</v>
       </c>
     </row>
@@ -25784,7 +25840,7 @@
       <c r="C41" s="80" t="s">
         <v>781</v>
       </c>
-      <c r="D41" s="476"/>
+      <c r="D41" s="453"/>
     </row>
     <row r="42" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B42" s="223" t="s">
@@ -25793,7 +25849,7 @@
       <c r="C42" s="80" t="s">
         <v>782</v>
       </c>
-      <c r="D42" s="476"/>
+      <c r="D42" s="453"/>
     </row>
     <row r="43" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B43" s="225" t="s">
@@ -25802,7 +25858,7 @@
       <c r="C43" s="227" t="s">
         <v>778</v>
       </c>
-      <c r="D43" s="477"/>
+      <c r="D43" s="454"/>
     </row>
     <row r="44" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="45" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -25820,17 +25876,17 @@
       <c r="B46" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C46" s="460" t="s">
+      <c r="C46" s="455" t="s">
         <v>668</v>
       </c>
-      <c r="D46" s="461"/>
+      <c r="D46" s="456"/>
     </row>
     <row r="47" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B47" s="304" t="s">
         <v>783</v>
       </c>
       <c r="C47" s="303"/>
-      <c r="D47" s="475"/>
+      <c r="D47" s="452"/>
     </row>
     <row r="48" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B48" s="223" t="s">
@@ -25839,7 +25895,7 @@
       <c r="C48" s="80" t="s">
         <v>787</v>
       </c>
-      <c r="D48" s="476"/>
+      <c r="D48" s="453"/>
     </row>
     <row r="49" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B49" s="225" t="s">
@@ -25848,7 +25904,7 @@
       <c r="C49" s="227" t="s">
         <v>786</v>
       </c>
-      <c r="D49" s="477"/>
+      <c r="D49" s="454"/>
     </row>
     <row r="50" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="51" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -25866,10 +25922,10 @@
       <c r="B52" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C52" s="460" t="s">
+      <c r="C52" s="455" t="s">
         <v>668</v>
       </c>
-      <c r="D52" s="461"/>
+      <c r="D52" s="456"/>
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B53" s="304" t="s">
@@ -25878,7 +25934,7 @@
       <c r="C53" s="303" t="s">
         <v>793</v>
       </c>
-      <c r="D53" s="475" t="s">
+      <c r="D53" s="452" t="s">
         <v>795</v>
       </c>
     </row>
@@ -25889,7 +25945,7 @@
       <c r="C54" s="80" t="s">
         <v>792</v>
       </c>
-      <c r="D54" s="476"/>
+      <c r="D54" s="453"/>
     </row>
     <row r="55" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B55" s="223" t="s">
@@ -25898,14 +25954,14 @@
       <c r="C55" s="80" t="s">
         <v>794</v>
       </c>
-      <c r="D55" s="476"/>
+      <c r="D55" s="453"/>
     </row>
     <row r="56" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B56" s="225" t="s">
         <v>791</v>
       </c>
       <c r="C56" s="227"/>
-      <c r="D56" s="477"/>
+      <c r="D56" s="454"/>
     </row>
     <row r="57" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="58" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -25923,290 +25979,290 @@
       <c r="B59" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C59" s="460" t="s">
+      <c r="C59" s="455" t="s">
         <v>668</v>
       </c>
-      <c r="D59" s="461"/>
+      <c r="D59" s="456"/>
     </row>
     <row r="60" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B60" s="304" t="s">
         <v>841</v>
       </c>
-      <c r="C60" s="454"/>
-      <c r="D60" s="455"/>
+      <c r="C60" s="465"/>
+      <c r="D60" s="466"/>
     </row>
     <row r="61" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B61" s="223" t="s">
         <v>842</v>
       </c>
-      <c r="C61" s="456"/>
-      <c r="D61" s="457"/>
+      <c r="C61" s="467"/>
+      <c r="D61" s="468"/>
     </row>
     <row r="62" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B62" s="223" t="s">
         <v>843</v>
       </c>
-      <c r="C62" s="456"/>
-      <c r="D62" s="457"/>
+      <c r="C62" s="467"/>
+      <c r="D62" s="468"/>
     </row>
     <row r="63" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B63" s="223" t="s">
         <v>844</v>
       </c>
-      <c r="C63" s="456"/>
-      <c r="D63" s="457"/>
+      <c r="C63" s="467"/>
+      <c r="D63" s="468"/>
     </row>
     <row r="64" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B64" s="223" t="s">
         <v>845</v>
       </c>
-      <c r="C64" s="456"/>
-      <c r="D64" s="457"/>
+      <c r="C64" s="467"/>
+      <c r="D64" s="468"/>
     </row>
     <row r="65" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B65" s="223" t="s">
         <v>846</v>
       </c>
-      <c r="C65" s="456"/>
-      <c r="D65" s="457"/>
+      <c r="C65" s="467"/>
+      <c r="D65" s="468"/>
     </row>
     <row r="66" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B66" s="223" t="s">
         <v>847</v>
       </c>
-      <c r="C66" s="456"/>
-      <c r="D66" s="457"/>
+      <c r="C66" s="467"/>
+      <c r="D66" s="468"/>
     </row>
     <row r="67" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B67" s="223" t="s">
         <v>848</v>
       </c>
-      <c r="C67" s="456"/>
-      <c r="D67" s="457"/>
+      <c r="C67" s="467"/>
+      <c r="D67" s="468"/>
     </row>
     <row r="68" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B68" s="223" t="s">
         <v>849</v>
       </c>
-      <c r="C68" s="456"/>
-      <c r="D68" s="457"/>
+      <c r="C68" s="467"/>
+      <c r="D68" s="468"/>
     </row>
     <row r="69" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B69" s="223" t="s">
         <v>850</v>
       </c>
-      <c r="C69" s="456"/>
-      <c r="D69" s="457"/>
+      <c r="C69" s="467"/>
+      <c r="D69" s="468"/>
     </row>
     <row r="70" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B70" s="223" t="s">
         <v>851</v>
       </c>
-      <c r="C70" s="456"/>
-      <c r="D70" s="457"/>
+      <c r="C70" s="467"/>
+      <c r="D70" s="468"/>
     </row>
     <row r="71" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B71" s="223" t="s">
         <v>852</v>
       </c>
-      <c r="C71" s="456"/>
-      <c r="D71" s="457"/>
+      <c r="C71" s="467"/>
+      <c r="D71" s="468"/>
     </row>
     <row r="72" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B72" s="223" t="s">
         <v>853</v>
       </c>
-      <c r="C72" s="456"/>
-      <c r="D72" s="457"/>
+      <c r="C72" s="467"/>
+      <c r="D72" s="468"/>
     </row>
     <row r="73" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B73" s="223" t="s">
         <v>854</v>
       </c>
-      <c r="C73" s="456"/>
-      <c r="D73" s="457"/>
+      <c r="C73" s="467"/>
+      <c r="D73" s="468"/>
     </row>
     <row r="74" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B74" s="223" t="s">
         <v>855</v>
       </c>
-      <c r="C74" s="456"/>
-      <c r="D74" s="457"/>
+      <c r="C74" s="467"/>
+      <c r="D74" s="468"/>
     </row>
     <row r="75" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B75" s="223" t="s">
         <v>856</v>
       </c>
-      <c r="C75" s="456"/>
-      <c r="D75" s="457"/>
+      <c r="C75" s="467"/>
+      <c r="D75" s="468"/>
     </row>
     <row r="76" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B76" s="223" t="s">
         <v>857</v>
       </c>
-      <c r="C76" s="456"/>
-      <c r="D76" s="457"/>
+      <c r="C76" s="467"/>
+      <c r="D76" s="468"/>
     </row>
     <row r="77" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B77" s="223" t="s">
         <v>858</v>
       </c>
-      <c r="C77" s="456"/>
-      <c r="D77" s="457"/>
+      <c r="C77" s="467"/>
+      <c r="D77" s="468"/>
     </row>
     <row r="78" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B78" s="223" t="s">
         <v>859</v>
       </c>
-      <c r="C78" s="456"/>
-      <c r="D78" s="457"/>
+      <c r="C78" s="467"/>
+      <c r="D78" s="468"/>
     </row>
     <row r="79" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B79" s="223" t="s">
         <v>860</v>
       </c>
-      <c r="C79" s="456"/>
-      <c r="D79" s="457"/>
+      <c r="C79" s="467"/>
+      <c r="D79" s="468"/>
     </row>
     <row r="80" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B80" s="223" t="s">
         <v>861</v>
       </c>
-      <c r="C80" s="456"/>
-      <c r="D80" s="457"/>
+      <c r="C80" s="467"/>
+      <c r="D80" s="468"/>
     </row>
     <row r="81" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B81" s="223" t="s">
         <v>862</v>
       </c>
-      <c r="C81" s="456"/>
-      <c r="D81" s="457"/>
+      <c r="C81" s="467"/>
+      <c r="D81" s="468"/>
     </row>
     <row r="82" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B82" s="223" t="s">
         <v>863</v>
       </c>
-      <c r="C82" s="456"/>
-      <c r="D82" s="457"/>
+      <c r="C82" s="467"/>
+      <c r="D82" s="468"/>
     </row>
     <row r="83" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B83" s="223" t="s">
         <v>864</v>
       </c>
-      <c r="C83" s="456"/>
-      <c r="D83" s="457"/>
+      <c r="C83" s="467"/>
+      <c r="D83" s="468"/>
     </row>
     <row r="84" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B84" s="223" t="s">
         <v>865</v>
       </c>
-      <c r="C84" s="456"/>
-      <c r="D84" s="457"/>
+      <c r="C84" s="467"/>
+      <c r="D84" s="468"/>
     </row>
     <row r="85" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B85" s="223" t="s">
         <v>866</v>
       </c>
-      <c r="C85" s="456"/>
-      <c r="D85" s="457"/>
+      <c r="C85" s="467"/>
+      <c r="D85" s="468"/>
     </row>
     <row r="86" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B86" s="223" t="s">
         <v>867</v>
       </c>
-      <c r="C86" s="456"/>
-      <c r="D86" s="457"/>
+      <c r="C86" s="467"/>
+      <c r="D86" s="468"/>
     </row>
     <row r="87" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B87" s="223" t="s">
         <v>868</v>
       </c>
-      <c r="C87" s="456"/>
-      <c r="D87" s="457"/>
+      <c r="C87" s="467"/>
+      <c r="D87" s="468"/>
     </row>
     <row r="88" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B88" s="223" t="s">
         <v>869</v>
       </c>
-      <c r="C88" s="456"/>
-      <c r="D88" s="457"/>
+      <c r="C88" s="467"/>
+      <c r="D88" s="468"/>
     </row>
     <row r="89" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B89" s="223" t="s">
         <v>870</v>
       </c>
-      <c r="C89" s="456"/>
-      <c r="D89" s="457"/>
+      <c r="C89" s="467"/>
+      <c r="D89" s="468"/>
     </row>
     <row r="90" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B90" s="223" t="s">
         <v>871</v>
       </c>
-      <c r="C90" s="456"/>
-      <c r="D90" s="457"/>
+      <c r="C90" s="467"/>
+      <c r="D90" s="468"/>
     </row>
     <row r="91" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B91" s="223" t="s">
         <v>872</v>
       </c>
-      <c r="C91" s="456"/>
-      <c r="D91" s="457"/>
+      <c r="C91" s="467"/>
+      <c r="D91" s="468"/>
     </row>
     <row r="92" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B92" s="223" t="s">
         <v>873</v>
       </c>
-      <c r="C92" s="456"/>
-      <c r="D92" s="457"/>
+      <c r="C92" s="467"/>
+      <c r="D92" s="468"/>
     </row>
     <row r="93" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B93" s="223" t="s">
         <v>874</v>
       </c>
-      <c r="C93" s="456"/>
-      <c r="D93" s="457"/>
+      <c r="C93" s="467"/>
+      <c r="D93" s="468"/>
     </row>
     <row r="94" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B94" s="223" t="s">
         <v>875</v>
       </c>
-      <c r="C94" s="456"/>
-      <c r="D94" s="457"/>
+      <c r="C94" s="467"/>
+      <c r="D94" s="468"/>
     </row>
     <row r="95" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B95" s="223" t="s">
         <v>876</v>
       </c>
-      <c r="C95" s="456"/>
-      <c r="D95" s="457"/>
+      <c r="C95" s="467"/>
+      <c r="D95" s="468"/>
     </row>
     <row r="96" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B96" s="223" t="s">
         <v>877</v>
       </c>
-      <c r="C96" s="456"/>
-      <c r="D96" s="457"/>
+      <c r="C96" s="467"/>
+      <c r="D96" s="468"/>
     </row>
     <row r="97" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B97" s="223" t="s">
         <v>878</v>
       </c>
-      <c r="C97" s="456"/>
-      <c r="D97" s="457"/>
+      <c r="C97" s="467"/>
+      <c r="D97" s="468"/>
     </row>
     <row r="98" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B98" s="223" t="s">
         <v>879</v>
       </c>
-      <c r="C98" s="456"/>
-      <c r="D98" s="457"/>
+      <c r="C98" s="467"/>
+      <c r="D98" s="468"/>
     </row>
     <row r="99" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B99" s="225" t="s">
         <v>880</v>
       </c>
-      <c r="C99" s="458"/>
-      <c r="D99" s="459"/>
+      <c r="C99" s="469"/>
+      <c r="D99" s="470"/>
     </row>
     <row r="100" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="101" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -26224,38 +26280,38 @@
       <c r="B102" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C102" s="460" t="s">
+      <c r="C102" s="455" t="s">
         <v>668</v>
       </c>
-      <c r="D102" s="461"/>
+      <c r="D102" s="456"/>
     </row>
     <row r="103" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B103" s="304" t="s">
         <v>881</v>
       </c>
-      <c r="C103" s="462"/>
-      <c r="D103" s="463"/>
+      <c r="C103" s="457"/>
+      <c r="D103" s="458"/>
     </row>
     <row r="104" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B104" s="223" t="s">
         <v>882</v>
       </c>
-      <c r="C104" s="464"/>
-      <c r="D104" s="465"/>
+      <c r="C104" s="459"/>
+      <c r="D104" s="460"/>
     </row>
     <row r="105" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B105" s="223" t="s">
         <v>883</v>
       </c>
-      <c r="C105" s="464"/>
-      <c r="D105" s="465"/>
+      <c r="C105" s="459"/>
+      <c r="D105" s="460"/>
     </row>
     <row r="106" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B106" s="225" t="s">
         <v>884</v>
       </c>
-      <c r="C106" s="466"/>
-      <c r="D106" s="467"/>
+      <c r="C106" s="461"/>
+      <c r="D106" s="462"/>
     </row>
     <row r="107" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="108" spans="2:4" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -26273,19 +26329,19 @@
       <c r="B109" s="312" t="s">
         <v>749</v>
       </c>
-      <c r="C109" s="460" t="s">
+      <c r="C109" s="455" t="s">
         <v>668</v>
       </c>
-      <c r="D109" s="461"/>
+      <c r="D109" s="456"/>
     </row>
     <row r="110" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B110" s="304" t="s">
         <v>803</v>
       </c>
-      <c r="C110" s="468" t="s">
+      <c r="C110" s="471" t="s">
         <v>682</v>
       </c>
-      <c r="D110" s="474" t="s">
+      <c r="D110" s="477" t="s">
         <v>817</v>
       </c>
     </row>
@@ -26293,94 +26349,94 @@
       <c r="B111" s="223" t="s">
         <v>804</v>
       </c>
-      <c r="C111" s="469"/>
-      <c r="D111" s="472"/>
+      <c r="C111" s="472"/>
+      <c r="D111" s="475"/>
     </row>
     <row r="112" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B112" s="223" t="s">
         <v>805</v>
       </c>
-      <c r="C112" s="469"/>
-      <c r="D112" s="472"/>
+      <c r="C112" s="472"/>
+      <c r="D112" s="475"/>
     </row>
     <row r="113" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B113" s="223" t="s">
         <v>806</v>
       </c>
-      <c r="C113" s="469"/>
-      <c r="D113" s="472"/>
+      <c r="C113" s="472"/>
+      <c r="D113" s="475"/>
     </row>
     <row r="114" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B114" s="223" t="s">
         <v>807</v>
       </c>
-      <c r="C114" s="469"/>
-      <c r="D114" s="472"/>
+      <c r="C114" s="472"/>
+      <c r="D114" s="475"/>
     </row>
     <row r="115" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B115" s="223" t="s">
         <v>808</v>
       </c>
-      <c r="C115" s="469"/>
-      <c r="D115" s="472"/>
+      <c r="C115" s="472"/>
+      <c r="D115" s="475"/>
     </row>
     <row r="116" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B116" s="223" t="s">
         <v>809</v>
       </c>
-      <c r="C116" s="469"/>
-      <c r="D116" s="472"/>
+      <c r="C116" s="472"/>
+      <c r="D116" s="475"/>
     </row>
     <row r="117" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B117" s="223" t="s">
         <v>810</v>
       </c>
-      <c r="C117" s="469"/>
-      <c r="D117" s="472"/>
+      <c r="C117" s="472"/>
+      <c r="D117" s="475"/>
     </row>
     <row r="118" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B118" s="223" t="s">
         <v>811</v>
       </c>
-      <c r="C118" s="469"/>
-      <c r="D118" s="472"/>
+      <c r="C118" s="472"/>
+      <c r="D118" s="475"/>
     </row>
     <row r="119" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B119" s="223" t="s">
         <v>812</v>
       </c>
-      <c r="C119" s="469"/>
-      <c r="D119" s="472"/>
+      <c r="C119" s="472"/>
+      <c r="D119" s="475"/>
     </row>
     <row r="120" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B120" s="223" t="s">
         <v>813</v>
       </c>
-      <c r="C120" s="470"/>
-      <c r="D120" s="472"/>
+      <c r="C120" s="473"/>
+      <c r="D120" s="475"/>
     </row>
     <row r="121" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B121" s="223" t="s">
         <v>814</v>
       </c>
-      <c r="C121" s="471" t="s">
+      <c r="C121" s="474" t="s">
         <v>683</v>
       </c>
-      <c r="D121" s="472"/>
+      <c r="D121" s="475"/>
     </row>
     <row r="122" spans="2:4" s="36" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B122" s="223" t="s">
         <v>815</v>
       </c>
-      <c r="C122" s="472"/>
-      <c r="D122" s="472"/>
+      <c r="C122" s="475"/>
+      <c r="D122" s="475"/>
     </row>
     <row r="123" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B123" s="225" t="s">
         <v>816</v>
       </c>
-      <c r="C123" s="473"/>
-      <c r="D123" s="473"/>
+      <c r="C123" s="476"/>
+      <c r="D123" s="476"/>
     </row>
     <row r="124" spans="2:4" s="36" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B124" s="240"/>
@@ -26402,22 +26458,36 @@
       <c r="B126" s="312" t="s">
         <v>819</v>
       </c>
-      <c r="C126" s="460" t="s">
+      <c r="C126" s="455" t="s">
         <v>668</v>
       </c>
-      <c r="D126" s="461"/>
+      <c r="D126" s="456"/>
     </row>
     <row r="127" spans="2:4" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B127" s="330" t="s">
         <v>818</v>
       </c>
-      <c r="C127" s="452" t="s">
+      <c r="C127" s="463" t="s">
         <v>820</v>
       </c>
-      <c r="D127" s="453"/>
+      <c r="D127" s="464"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="C127:D127"/>
+    <mergeCell ref="C60:D99"/>
+    <mergeCell ref="C102:D102"/>
+    <mergeCell ref="C103:D106"/>
+    <mergeCell ref="C109:D109"/>
+    <mergeCell ref="C126:D126"/>
+    <mergeCell ref="C110:C120"/>
+    <mergeCell ref="C121:C123"/>
+    <mergeCell ref="D110:D123"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="D47:D49"/>
+    <mergeCell ref="C52:D52"/>
+    <mergeCell ref="D53:D56"/>
+    <mergeCell ref="C59:D59"/>
     <mergeCell ref="D40:D43"/>
     <mergeCell ref="D6:D10"/>
     <mergeCell ref="C5:D5"/>
@@ -26428,20 +26498,6 @@
     <mergeCell ref="C27:D27"/>
     <mergeCell ref="C28:D36"/>
     <mergeCell ref="C39:D39"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="D47:D49"/>
-    <mergeCell ref="C52:D52"/>
-    <mergeCell ref="D53:D56"/>
-    <mergeCell ref="C59:D59"/>
-    <mergeCell ref="C127:D127"/>
-    <mergeCell ref="C60:D99"/>
-    <mergeCell ref="C102:D102"/>
-    <mergeCell ref="C103:D106"/>
-    <mergeCell ref="C109:D109"/>
-    <mergeCell ref="C126:D126"/>
-    <mergeCell ref="C110:C120"/>
-    <mergeCell ref="C121:C123"/>
-    <mergeCell ref="D110:D123"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>